<commit_message>
Balanceia os ciclos de prestígio e o preço dos recrutas de nível alto
Closes #44
</commit_message>
<xml_diff>
--- a/docs/balanceamento/Balanceamento_v1.xlsx
+++ b/docs/balanceamento/Balanceamento_v1.xlsx
@@ -873,7 +873,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>1.8</v>
+        <v>6</v>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
@@ -948,7 +948,7 @@
         </is>
       </c>
       <c r="B21" s="6" t="n">
-        <v>1.25</v>
+        <v>1.12</v>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
@@ -978,7 +978,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>1.1</v>
+        <v>1.05</v>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>

</xml_diff>